<commit_message>
Few changes on DDT Cases
</commit_message>
<xml_diff>
--- a/TestData/SpiceClub.xlsx
+++ b/TestData/SpiceClub.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/saidharmarajuboina/eclipse-workspace/AutomationConcepts1/TestData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A57DFA3F-9F18-8E4C-856C-BFD55FB26F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9D02603-18D5-6547-95CB-D0681202B042}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17880" activeTab="1" xr2:uid="{8EEDDA7D-502D-6B4E-B9F9-8EDFEAE67728}"/>
+    <workbookView xWindow="4420" yWindow="660" windowWidth="25820" windowHeight="17880" xr2:uid="{8EEDDA7D-502D-6B4E-B9F9-8EDFEAE67728}"/>
   </bookViews>
   <sheets>
     <sheet name="SignUp" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>First Name and Middle Name*</t>
   </si>
@@ -112,9 +112,6 @@
   </si>
   <si>
     <t>PassSpice1$$$$$</t>
-  </si>
-  <si>
-    <t>User6FName</t>
   </si>
   <si>
     <t>User6lName</t>
@@ -622,17 +619,14 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" t="s">
+      <c r="B7" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="C7" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" t="s">
         <v>25</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>